<commit_message>
sync: Live-Verify-Ergebnisse in Tools + Handover + Faktortabelle eingepflegt
Satelliten_Monitor S-Spalte (Hinweis): LV-Notizen für ASML/TMO/RMS angehängt inkl. Watch-Hinweis ASML Fwd P/E FY27 30,30 Grenzfall.

SESSION-HANDOVER: Backtest-Tabelle um Live-Verify-Spalte erweitert (✅ 3/11 verifiziert, ⏳ 8 offen bei Earnings-Trigger). Differenzierung Fix-1 (TMO nur P/FCF) vs. maximal (ASML/RMS beide Zweige) dokumentiert.

Faktortabelle: Info-Note um Live-Verify-Status ergänzt.

Keine Score-/DEFCON-/Sparraten-Korrekturen nötig — Approximationen innerhalb ±2 Toleranz bestätigt.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Satelliten_Monitor_v2.0.xlsx
+++ b/03_Tools/Satelliten_Monitor_v2.0.xlsx
@@ -993,7 +993,7 @@
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>[V] DEFCON 3 (68/100). Moat 19/20 Wide Monopol, Fwd P/E 38x + P/FCF ~41x = Bewertungsprämie ohne Sicherheitsmarge. China-Revenue 14.7% → Kein Tariff-FLAG.</t>
+          <t>[V] DEFCON 3 (68/100). Moat 19/20 Wide Monopol, Fwd P/E 38x + P/FCF ~41x = Bewertungsprämie ohne Sicherheitsmarge. China-Revenue 14.7% → Kein Tariff-FLAG.  |  [LV 17.04.] v3.7 Live-Verify: Score 66 ±2 bestätigt (OpM 36,1% / Fwd P/E 39,52 + P/FCF 48x → beide Fix-1-Zweige hart 0). WATCH: Fwd P/E FY27 30,30 Grenzfall — bei &lt;30 nach Guidance Score +1-2 (D4-Upside).</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>[V] Re-Analyse 15.04.2026: Score 71→69 (−2). Q1 2026: €4.07B (+6% CER, −1% reported). Miss vs. +7–8% Konsens. Kursreaktion −8.4% (€1.783→€1.632,50). 52W-Tief €1.529 intraday. Treiber: Mittlerer Osten −6% (Iran-Krieg, UAE Malls −40%), FX-Headwind €290M, China +2%. Positiv: Leder +9%, ROIC 24%&gt;&gt;WACC 6.5%, Insider Buy +€7.67M (AMF). Kein FLAG. Sparplan voll aktiv. Nächster Check: H1 2026 Report.</t>
+          <t>[V] Re-Analyse 15.04.2026: Score 71→69 (−2). Q1 2026: €4.07B (+6% CER, −1% reported). Miss vs. +7–8% Konsens. Kursreaktion −8.4% (€1.783→€1.632,50). 52W-Tief €1.529 intraday. Treiber: Mittlerer Osten −6% (Iran-Krieg, UAE Malls −40%), FX-Headwind €290M, China +2%. Positiv: Leder +9%, ROIC 24%&gt;&gt;WACC 6.5%, Insider Buy +€7.67M (AMF). Kein FLAG. Sparplan voll aktiv. Nächster Check: H1 2026 Report.  |  [LV 17.04.] v3.7 Live-Verify: Score 68 ±2 bestätigt (OpM 41,05% / Fwd P/E 34,91 + P/FCF 38x → beide Fix-1-Zweige hart 0). D4 durch Screener-Exception (ROIC 24% &gt;&gt; WACC +17,5pp) geschützt. Nach −8,4% Kursdrop Fwd P/E von 39→34,9.</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="S16" s="10" t="inlineStr">
         <is>
-          <t>[V] Re-Analyse 07.04.: Score 65→67 (+2). Net Debt/EBITDA 3.6x→2.57x ✅. Fwd P/E 27x→19.9x ✅. ROIC 2.6% &lt; WACC bleibt Schwäche. FCF −13.4% YoY. Trigger 23.04.: FCF &gt;.3B nötig.</t>
+          <t>[V] Re-Analyse 07.04.: Score 65→67 (+2). Net Debt/EBITDA 3.6x→2.57x ✅. Fwd P/E 27x→19.9x ✅. ROIC 2.6% &lt; WACC bleibt Schwäche. FCF −13.4% YoY. Trigger 23.04.: FCF &gt;.3B nötig.  |  [LV 17.04.] v3.7 Live-Verify: Score 63 ±1 bestätigt (OpM 18,17% / Fwd P/E FY26 20,80 unter Schwelle → nur P/FCF 29,3x triggert Fix-1). Sell-Ratio 0% Warning. Q1 Earnings 23.04. kritisch.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync(flag): AVGO Insider-FLAG Kaskade in XLSX-Tools (Rebalancing + Satelliten-Monitor)
- Rebalancing_Tool_v3.4.xlsx: A2 Stand 28.04., O11 (AVGO FLAG-Status) "✅ Clean" → "🔴 FLAG: Insider-Selling 90d $106M+ | Aktiviert 27.04.2026 | Re-Eval Q3 FY26". Sparrate-Formeln (P-Spalte) rechnen Nenner 8.5→7.5 + Sparraten automatisch nach (LEFT(O,1)="🔴" Trigger greift).
- Satelliten_Monitor_v2.0.xlsx: O2 Stand 28.04., H3 Eingefroren-Liste um AVGO erweitert, K3 Zähler 8/1/2 → 7/1/3, R8 (AVGO) Sparrate 33.53→0 + Status-Text. 7 D3/D4-Satelliten Sparrate 33.53→38.00 (R7/R10/R11/R12/R13/R14/R16, plus N-Text 33,53€→38,00€). V D2 Sparrate 16.76→19.00.
- STATE.md Last-Audit-Timestamp-Refresh.

User-Aktion fertig — beide XLSX-Tools matchen jetzt config.yaml/PORTFOLIO.md/Faktortabelle.md.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Satelliten_Monitor_v2.0.xlsx
+++ b/03_Tools/Satelliten_Monitor_v2.0.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Satelliten Monitor" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="QuickScreen Ampel" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Satelliten Monitor" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuickScreen Ampel" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -833,7 +833,7 @@
       </c>
       <c r="O2" s="31" t="inlineStr">
         <is>
-          <t>Stand: 23.04.2026  |  Broker: Scalable Capital  |  Slots: 11/11</t>
+          <t>Stand: 28.04.2026  |  Broker: Scalable Capital  |  Slots: 11/11</t>
         </is>
       </c>
     </row>
@@ -850,12 +850,12 @@
       </c>
       <c r="H3" s="33" t="inlineStr">
         <is>
-          <t>Eingefroren: MSFT (🔴 FLAG CapEx/OCF, D2) | APH (🔴 FLAG Score-basiert, D2 seit 18.04.) — Sparrate 0€</t>
+          <t>Eingefroren: MSFT (🔴 CapEx/OCF &gt;60%, D2) | APH (🔴 Score-basiert, D2) | AVGO (🔴 Insider-Selling 90d $106M+, ab 27.04.) — Sparrate 0€</t>
         </is>
       </c>
       <c r="K3" s="33" t="inlineStr">
         <is>
-          <t>Ergebnis: 🟢 8 Voll  🟠 1 D2-Sockelbetrag (V)  🔴 2 Eingefroren (MSFT, APH)</t>
+          <t>Ergebnis: 🟢 7 Voll  🟠 1 D2-Sockelbetrag (V)  🔴 3 Eingefroren (MSFT, APH, AVGO)</t>
         </is>
       </c>
       <c r="N3" s="34" t="inlineStr">
@@ -1044,11 +1044,11 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>🟡 DEFCON 3 / ✅ Volle Rate 33,53€ (D3=1.0, Nenner 8.5 post-TMO-Q1)</t>
+          <t>🟡 DEFCON 3 / ✅ Volle Rate 38,00€ (D3=1.0, Nenner 7.5 post-TMO-Q1)</t>
         </is>
       </c>
       <c r="O7" s="8" t="n">
-        <v>33.53</v>
+        <v>38</v>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
@@ -1131,11 +1131,11 @@
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>⚠️ Insider-Check ausstehend (verm. Post-Vesting) | Sparplan läuft</t>
+          <t>🔴 FLAG: Insider-Selling 90d $106M+ (5-14× Schwelle) | OpenInsider 9 Tx „S - Sale" ohne 10b5-1-Suffix | Aktiviert 27.04.2026 | Re-Eval Q3 FY26</t>
         </is>
       </c>
       <c r="O8" s="8" t="n">
-        <v>33.53</v>
+        <v>0</v>
       </c>
       <c r="P8" s="11" t="inlineStr">
         <is>
@@ -1309,7 +1309,7 @@
         </is>
       </c>
       <c r="O10" s="8" t="n">
-        <v>33.53</v>
+        <v>38</v>
       </c>
       <c r="P10" s="11" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
         </is>
       </c>
       <c r="O11" s="8" t="n">
-        <v>33.53</v>
+        <v>38</v>
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
         </is>
       </c>
       <c r="O12" s="8" t="n">
-        <v>33.53</v>
+        <v>38</v>
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="O13" s="8" t="n">
-        <v>33.53</v>
+        <v>38</v>
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="O14" s="8" t="n">
-        <v>33.53</v>
+        <v>38</v>
       </c>
       <c r="P14" s="11" t="inlineStr">
         <is>
@@ -1740,11 +1740,11 @@
       </c>
       <c r="N15" s="13" t="inlineStr">
         <is>
-          <t>🟠 DEFCON 2 / ⏸ Sockelbetrag 16,76€ | Forward 18.04. nach Advisor-Review | Q2 FY26 28.04.</t>
+          <t>🟠 DEFCON 2 / ⏸ Sockelbetrag 19,00€ | Forward 18.04. nach Advisor-Review | Q2 FY26 28.04.</t>
         </is>
       </c>
       <c r="O15" s="8" t="n">
-        <v>16.76</v>
+        <v>19</v>
       </c>
       <c r="P15" s="5" t="inlineStr">
         <is>
@@ -1827,11 +1827,11 @@
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>🟡 DEFCON 3 / ✅ Volle Rate 33,53€ | fcf_trend_neg Resolve (Q1 WC-Unwind) | Q2 ~Ende Juli</t>
+          <t>🟡 DEFCON 3 / ✅ Volle Rate 38,00€ | fcf_trend_neg Resolve (Q1 WC-Unwind) | Q2 ~Ende Juli</t>
         </is>
       </c>
       <c r="O16" s="15" t="n">
-        <v>33.53</v>
+        <v>38</v>
       </c>
       <c r="P16" s="11" t="inlineStr">
         <is>

</xml_diff>